<commit_message>
feat(admin/finalexams)#001: Complete 3 helpers for Course Module and 2 func for exam manager (Service and Repository pattern only)
</commit_message>
<xml_diff>
--- a/Document/Bao_cao_tien_do_15052026.xlsx
+++ b/Document/Bao_cao_tien_do_15052026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\for_Work\TPS_FullStack\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411CD383-6176-4E8C-B99F-0B7C17D563D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE8882D-8BA4-4BA0-B306-B315959E65B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{71C6B39C-7555-4D73-AEC4-4EDB26693EEC}"/>
+    <workbookView xWindow="10515" yWindow="0" windowWidth="18390" windowHeight="15585" xr2:uid="{71C6B39C-7555-4D73-AEC4-4EDB26693EEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Database - Giải thích " sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="262">
   <si>
     <t>Danh sách các bảng database</t>
   </si>
@@ -823,12 +823,129 @@
 Test case thoả khi thực hiện upgrade logic:
 - Thu: 2#4#6, Ngaybatdau: 12/05/2026</t>
   </si>
+  <si>
+    <t>decimal(5,2)</t>
+  </si>
+  <si>
+    <t>Thoigianlambai</t>
+  </si>
+  <si>
+    <t>BaithuhoachID</t>
+  </si>
+  <si>
+    <t>TraloiID</t>
+  </si>
+  <si>
+    <t>DapanID</t>
+  </si>
+  <si>
+    <t>Baithuhoach</t>
+  </si>
+  <si>
+    <t>Baithuhoach_Cauhoi</t>
+  </si>
+  <si>
+    <t>Ghi nhận thời gian làm bài của học viên</t>
+  </si>
+  <si>
+    <t>Ghi nhận câu trả lời của học viên</t>
+  </si>
+  <si>
+    <t>Đáp án đúng</t>
+  </si>
+  <si>
+    <t>Ghi nhận đúng sai của câu trả lời</t>
+  </si>
+  <si>
+    <t>Module giảng viên</t>
+  </si>
+  <si>
+    <t>api/teacher/Teacher/information/{teacherId}</t>
+  </si>
+  <si>
+    <t>api/teacher/Teacher/schedules/{teacherId}</t>
+  </si>
+  <si>
+    <t>api/teacher/Teacher/attendance</t>
+  </si>
+  <si>
+    <t>api/student/info/{MaID}</t>
+  </si>
+  <si>
+    <t>api/student/schedule/{MaID}</t>
+  </si>
+  <si>
+    <t>api/student/checkin</t>
+  </si>
+  <si>
+    <t>api/student/courses/{MaID}</t>
+  </si>
+  <si>
+    <t>/api/student/courseinfo/{MaID}/{KhoahocID}</t>
+  </si>
+  <si>
+    <t>Module học viên</t>
+  </si>
+  <si>
+    <t>Thông tin giảng viên</t>
+  </si>
+  <si>
+    <t>Lịch dạy/ Thời khóa biểu giảng viên</t>
+  </si>
+  <si>
+    <t>Điểm danh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thông tin học viên </t>
+  </si>
+  <si>
+    <t>Lịch học/ Thời khóa biểu học viên</t>
+  </si>
+  <si>
+    <t>Danh sách khóa học (lọc theo HocvienID)</t>
+  </si>
+  <si>
+    <t>Thông tin chi tiết khóa học</t>
+  </si>
+  <si>
+    <t>Nộp bài thu hoạch</t>
+  </si>
+  <si>
+    <t>Tạo bài thu hoạch</t>
+  </si>
+  <si>
+    <t>teacherId - string</t>
+  </si>
+  <si>
+    <t>lichhocID, hocvienID, khoahocID</t>
+  </si>
+  <si>
+    <t>MaID, KhoahocID</t>
+  </si>
+  <si>
+    <t>lichhocID, giangvienID, khoahocID</t>
+  </si>
+  <si>
+    <t>Giangvien, Chiuyende, Khoahoc, Lichhoc</t>
+  </si>
+  <si>
+    <t>Lichhoc_Giangvien_Diemdanh, Lichhoc</t>
+  </si>
+  <si>
+    <t>Hocvien,  Chungchi, Khoahoc</t>
+  </si>
+  <si>
+    <t>Khoahoc,  Khoahoc_Hocvien</t>
+  </si>
+  <si>
+    <t>Khoahoc, Chuyende, Chuyende_Tailieu</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -876,6 +993,13 @@
     <font>
       <b/>
       <sz val="15"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -954,16 +1078,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -973,21 +1091,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -998,23 +1114,47 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1603,8 +1743,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C91616B9-703D-4149-B4F7-04E1005070EB}">
-  <dimension ref="A4:E134"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A4:E152"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
     <col min="2" max="2" width="29.5703125" customWidth="1"/>
@@ -1613,1528 +1753,1754 @@
     <col min="5" max="5" width="67.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:5" ht="19.5">
+    <row r="4" spans="1:5" ht="19.5" x14ac:dyDescent="0.3">
       <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75">
-      <c r="A7" s="8">
+    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="9"/>
-    </row>
-    <row r="8" spans="1:5" ht="15.75">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="6" t="s">
+      <c r="D7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:5" ht="15.75">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="6" t="s">
+      <c r="D8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:5" ht="15.75">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="6" t="s">
+      <c r="E9" s="6"/>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="9"/>
-    </row>
-    <row r="11" spans="1:5" ht="15.75">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="6" t="s">
+      <c r="E10" s="6"/>
+    </row>
+    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="9"/>
-    </row>
-    <row r="12" spans="1:5" ht="15.75">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="6" t="s">
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="9"/>
-    </row>
-    <row r="13" spans="1:5" ht="15.75">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="6" t="s">
+      <c r="E12" s="6"/>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="9"/>
-    </row>
-    <row r="14" spans="1:5" ht="15.75">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="6" t="s">
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" ht="15.75">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="6" t="s">
+      <c r="E14" s="6"/>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="9"/>
-    </row>
-    <row r="16" spans="1:5" ht="15.75">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="6" t="s">
+      <c r="E15" s="6"/>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="9"/>
-    </row>
-    <row r="17" spans="1:5" ht="15.75">
-      <c r="A17" s="8">
+      <c r="E16" s="6"/>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="18">
         <v>2</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="9"/>
-    </row>
-    <row r="18" spans="1:5" ht="15.75">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="6" t="s">
+      <c r="D17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="9"/>
-    </row>
-    <row r="19" spans="1:5" ht="15.75">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="6" t="s">
+      <c r="D18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="6"/>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="9"/>
-    </row>
-    <row r="20" spans="1:5" ht="15.75">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="6" t="s">
+      <c r="E19" s="6"/>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="9"/>
-    </row>
-    <row r="21" spans="1:5" ht="15.75">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="6" t="s">
+      <c r="E20" s="6"/>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="9"/>
-    </row>
-    <row r="22" spans="1:5" ht="15.75">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="6" t="s">
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="9"/>
-    </row>
-    <row r="23" spans="1:5" ht="15.75">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="6" t="s">
+      <c r="E22" s="6"/>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="9"/>
-    </row>
-    <row r="24" spans="1:5" ht="15.75">
-      <c r="A24" s="8">
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="18">
         <v>3</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" s="9"/>
-    </row>
-    <row r="25" spans="1:5" ht="15.75">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="6" t="s">
+      <c r="D24" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="9"/>
-    </row>
-    <row r="26" spans="1:5" ht="15.75">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="6" t="s">
+      <c r="D25" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="6"/>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="9"/>
-    </row>
-    <row r="27" spans="1:5" ht="15.75">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="6" t="s">
+      <c r="E26" s="6"/>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="18"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E27" s="9"/>
-    </row>
-    <row r="28" spans="1:5" ht="15.75">
-      <c r="A28" s="8">
+      <c r="E27" s="6"/>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="18">
         <v>4</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E28" s="9"/>
-    </row>
-    <row r="29" spans="1:5" ht="15.75">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="6" t="s">
+      <c r="D28" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="6"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="18"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E29" s="9"/>
-    </row>
-    <row r="30" spans="1:5" ht="15.75">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="6" t="s">
+      <c r="D29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="6"/>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="18"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E30" s="9"/>
-    </row>
-    <row r="31" spans="1:5" ht="15.75">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="6" t="s">
+      <c r="D30" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="6"/>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="18"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E31" s="9"/>
-    </row>
-    <row r="32" spans="1:5" ht="15.75">
-      <c r="A32" s="8"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="6" t="s">
+      <c r="E31" s="6"/>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="18"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E32" s="9"/>
-    </row>
-    <row r="33" spans="1:5" ht="15.75">
-      <c r="A33" s="8">
+      <c r="E32" s="6"/>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="18">
         <v>5</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E33" s="9"/>
-    </row>
-    <row r="34" spans="1:5" ht="15.75">
-      <c r="A34" s="8"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="6" t="s">
+      <c r="D33" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" s="6"/>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="18"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D34" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E34" s="9"/>
-    </row>
-    <row r="35" spans="1:5" ht="15.75">
-      <c r="A35" s="8"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="6" t="s">
+      <c r="D34" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="6"/>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="18"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D35" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E35" s="9"/>
-    </row>
-    <row r="36" spans="1:5" ht="15.75">
-      <c r="A36" s="8">
+      <c r="D35" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E35" s="6"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="18">
         <v>6</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D36" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E36" s="9"/>
-    </row>
-    <row r="37" spans="1:5" ht="15.75">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="6" t="s">
+      <c r="D36" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E36" s="6"/>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E37" s="9" t="s">
+      <c r="E37" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15.75">
-      <c r="A38" s="8"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="6" t="s">
+    <row r="38" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="18"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E38" s="9"/>
-    </row>
-    <row r="39" spans="1:5" ht="15.75">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="6" t="s">
+      <c r="E38" s="6"/>
+    </row>
+    <row r="39" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="18"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D39" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="9"/>
-    </row>
-    <row r="40" spans="1:5" ht="15.75">
-      <c r="A40" s="8"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="6" t="s">
+      <c r="E39" s="6"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="18"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="D40" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15.75">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="6" t="s">
+    <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="18"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E41" s="9"/>
-    </row>
-    <row r="42" spans="1:5" ht="15.75">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="6" t="s">
+      <c r="D41" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E41" s="6"/>
+    </row>
+    <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="18"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D42" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E42" s="9"/>
-    </row>
-    <row r="43" spans="1:5" ht="15.75">
-      <c r="A43" s="8"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="6" t="s">
+      <c r="E42" s="6"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="18"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E43" s="9"/>
-    </row>
-    <row r="44" spans="1:5" ht="15.75">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="6" t="s">
+      <c r="D43" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43" s="6"/>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D44" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E44" s="9"/>
-    </row>
-    <row r="45" spans="1:5" ht="15.75">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="6" t="s">
+      <c r="E44" s="6"/>
+    </row>
+    <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="18"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E45" s="9"/>
-    </row>
-    <row r="46" spans="1:5" ht="15.75">
-      <c r="A46" s="8"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="6" t="s">
+      <c r="E45" s="6"/>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D46" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E46" s="9"/>
-    </row>
-    <row r="47" spans="1:5" ht="15.75">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="6" t="s">
+      <c r="E46" s="6"/>
+    </row>
+    <row r="47" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="D47" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E47" s="9"/>
-    </row>
-    <row r="48" spans="1:5" ht="15.75">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="6" t="s">
+      <c r="E47" s="6"/>
+    </row>
+    <row r="48" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E48" s="9"/>
-    </row>
-    <row r="49" spans="1:5" ht="15.75">
-      <c r="A49" s="8"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="6" t="s">
+      <c r="E48" s="6"/>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="18"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E49" s="9"/>
-    </row>
-    <row r="50" spans="1:5" ht="15.75">
-      <c r="A50" s="8"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="6" t="s">
+      <c r="E49" s="6"/>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="18"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E50" s="9"/>
-    </row>
-    <row r="51" spans="1:5" ht="15.75">
-      <c r="A51" s="8">
+      <c r="E50" s="6"/>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="18">
         <v>7</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D51" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E51" s="9"/>
-    </row>
-    <row r="52" spans="1:5" ht="15.75">
-      <c r="A52" s="8"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="6" t="s">
+      <c r="D51" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E51" s="6"/>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="18"/>
+      <c r="B52" s="18"/>
+      <c r="C52" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D52" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E52" s="9" t="s">
+      <c r="E52" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.75">
-      <c r="A53" s="8"/>
-      <c r="B53" s="8"/>
-      <c r="C53" s="6" t="s">
+    <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="18"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D53" s="6" t="s">
+      <c r="D53" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E53" s="9"/>
-    </row>
-    <row r="54" spans="1:5" ht="15.75">
-      <c r="A54" s="8"/>
-      <c r="B54" s="8"/>
-      <c r="C54" s="6" t="s">
+      <c r="E53" s="6"/>
+    </row>
+    <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A54" s="18"/>
+      <c r="B54" s="18"/>
+      <c r="C54" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D54" s="6" t="s">
+      <c r="D54" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E54" s="9"/>
-    </row>
-    <row r="55" spans="1:5" ht="15.75">
-      <c r="A55" s="8"/>
-      <c r="B55" s="8"/>
-      <c r="C55" s="6" t="s">
+      <c r="E54" s="6"/>
+    </row>
+    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A55" s="18"/>
+      <c r="B55" s="18"/>
+      <c r="C55" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D55" s="6" t="s">
+      <c r="D55" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E55" s="9"/>
-    </row>
-    <row r="56" spans="1:5" ht="15.75">
-      <c r="A56" s="8"/>
-      <c r="B56" s="8"/>
-      <c r="C56" s="6" t="s">
+      <c r="E55" s="6"/>
+    </row>
+    <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A56" s="18"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D56" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E56" s="9"/>
-    </row>
-    <row r="57" spans="1:5" ht="15.75">
-      <c r="A57" s="8"/>
-      <c r="B57" s="8"/>
-      <c r="C57" s="6" t="s">
+      <c r="D56" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E56" s="6"/>
+    </row>
+    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A57" s="18"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D57" s="6" t="s">
+      <c r="D57" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E57" s="9"/>
-    </row>
-    <row r="58" spans="1:5" ht="15.75">
-      <c r="A58" s="8"/>
-      <c r="B58" s="8"/>
-      <c r="C58" s="6" t="s">
+      <c r="E57" s="6"/>
+    </row>
+    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A58" s="18"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D58" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E58" s="9"/>
-    </row>
-    <row r="59" spans="1:5" ht="15.75">
-      <c r="A59" s="8"/>
-      <c r="B59" s="8"/>
-      <c r="C59" s="6" t="s">
+      <c r="D58" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E58" s="6"/>
+    </row>
+    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A59" s="18"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D59" s="6" t="s">
+      <c r="D59" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E59" s="9"/>
-    </row>
-    <row r="60" spans="1:5" ht="15.75">
-      <c r="A60" s="8"/>
-      <c r="B60" s="8"/>
-      <c r="C60" s="6" t="s">
+      <c r="E59" s="6"/>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A60" s="18"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D60" s="6" t="s">
+      <c r="D60" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E60" s="9"/>
-    </row>
-    <row r="61" spans="1:5" ht="15.75">
-      <c r="A61" s="8"/>
-      <c r="B61" s="8"/>
-      <c r="C61" s="6" t="s">
+      <c r="E60" s="6"/>
+    </row>
+    <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A61" s="18"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D61" s="6" t="s">
+      <c r="D61" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E61" s="9"/>
-    </row>
-    <row r="62" spans="1:5" ht="15.75">
-      <c r="A62" s="8"/>
-      <c r="B62" s="8"/>
-      <c r="C62" s="6" t="s">
+      <c r="E61" s="6"/>
+    </row>
+    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="18"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D62" s="6" t="s">
+      <c r="D62" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E62" s="9"/>
-    </row>
-    <row r="63" spans="1:5" ht="15.75">
-      <c r="A63" s="8"/>
-      <c r="B63" s="8"/>
-      <c r="C63" s="6" t="s">
+      <c r="E62" s="6"/>
+    </row>
+    <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A63" s="18"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D63" s="6" t="s">
+      <c r="D63" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E63" s="9"/>
-    </row>
-    <row r="64" spans="1:5" ht="15.75">
-      <c r="A64" s="8"/>
-      <c r="B64" s="8"/>
-      <c r="C64" s="6" t="s">
+      <c r="E63" s="6"/>
+    </row>
+    <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A64" s="18"/>
+      <c r="B64" s="18"/>
+      <c r="C64" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D64" s="6" t="s">
+      <c r="D64" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E64" s="9"/>
-    </row>
-    <row r="65" spans="1:5" ht="15.75">
-      <c r="A65" s="8"/>
-      <c r="B65" s="8"/>
-      <c r="C65" s="6" t="s">
+      <c r="E64" s="6"/>
+    </row>
+    <row r="65" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A65" s="18"/>
+      <c r="B65" s="18"/>
+      <c r="C65" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D65" s="6" t="s">
+      <c r="D65" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E65" s="9"/>
-    </row>
-    <row r="66" spans="1:5" ht="15.75">
-      <c r="A66" s="8">
+      <c r="E65" s="6"/>
+    </row>
+    <row r="66" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="18">
         <v>8</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="B66" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E66" s="9"/>
-    </row>
-    <row r="67" spans="1:5" ht="15.75">
-      <c r="A67" s="8"/>
-      <c r="B67" s="8"/>
-      <c r="C67" s="6" t="s">
+      <c r="D66" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E66" s="6"/>
+    </row>
+    <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="18"/>
+      <c r="B67" s="18"/>
+      <c r="C67" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D67" s="6" t="s">
+      <c r="D67" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E67" s="9"/>
-    </row>
-    <row r="68" spans="1:5" ht="15.75">
-      <c r="A68" s="8"/>
-      <c r="B68" s="8"/>
-      <c r="C68" s="6" t="s">
+      <c r="E67" s="6"/>
+    </row>
+    <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A68" s="18"/>
+      <c r="B68" s="18"/>
+      <c r="C68" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D68" s="6" t="s">
+      <c r="D68" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E68" s="9"/>
-    </row>
-    <row r="69" spans="1:5" ht="15.75">
-      <c r="A69" s="8"/>
-      <c r="B69" s="8"/>
-      <c r="C69" s="6" t="s">
+      <c r="E68" s="6"/>
+    </row>
+    <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A69" s="18"/>
+      <c r="B69" s="18"/>
+      <c r="C69" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D69" s="6" t="s">
+      <c r="D69" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E69" s="9"/>
-    </row>
-    <row r="70" spans="1:5" ht="15.75">
-      <c r="A70" s="8"/>
-      <c r="B70" s="8"/>
-      <c r="C70" s="6" t="s">
+      <c r="E69" s="6"/>
+    </row>
+    <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A70" s="18"/>
+      <c r="B70" s="18"/>
+      <c r="C70" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D70" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E70" s="9"/>
-    </row>
-    <row r="71" spans="1:5" ht="15.75">
-      <c r="A71" s="8"/>
-      <c r="B71" s="8"/>
-      <c r="C71" s="6" t="s">
+      <c r="D70" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E70" s="6"/>
+    </row>
+    <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A71" s="18"/>
+      <c r="B71" s="18"/>
+      <c r="C71" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D71" s="6" t="s">
+      <c r="D71" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E71" s="9"/>
-    </row>
-    <row r="72" spans="1:5" ht="15.75">
-      <c r="A72" s="8"/>
-      <c r="B72" s="8"/>
-      <c r="C72" s="6" t="s">
+      <c r="E71" s="6"/>
+    </row>
+    <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A72" s="18"/>
+      <c r="B72" s="18"/>
+      <c r="C72" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D72" s="6" t="s">
+      <c r="D72" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E72" s="9"/>
-    </row>
-    <row r="73" spans="1:5" ht="15.75">
-      <c r="A73" s="8"/>
-      <c r="B73" s="8"/>
-      <c r="C73" s="6" t="s">
+      <c r="E72" s="6"/>
+    </row>
+    <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A73" s="18"/>
+      <c r="B73" s="18"/>
+      <c r="C73" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D73" s="6" t="s">
+      <c r="D73" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E73" s="9"/>
-    </row>
-    <row r="74" spans="1:5" ht="15.75">
-      <c r="A74" s="8"/>
-      <c r="B74" s="8"/>
-      <c r="C74" s="6" t="s">
+      <c r="E73" s="6"/>
+    </row>
+    <row r="74" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A74" s="18"/>
+      <c r="B74" s="18"/>
+      <c r="C74" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D74" s="6" t="s">
+      <c r="D74" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E74" s="9"/>
-    </row>
-    <row r="75" spans="1:5" ht="15.75">
-      <c r="A75" s="8"/>
-      <c r="B75" s="8"/>
-      <c r="C75" s="6" t="s">
+      <c r="E74" s="6"/>
+    </row>
+    <row r="75" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A75" s="18"/>
+      <c r="B75" s="18"/>
+      <c r="C75" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D75" s="6" t="s">
+      <c r="D75" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E75" s="9"/>
-    </row>
-    <row r="76" spans="1:5" ht="15.75">
-      <c r="A76" s="8"/>
-      <c r="B76" s="8"/>
-      <c r="C76" s="6" t="s">
+      <c r="E75" s="6"/>
+    </row>
+    <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A76" s="18"/>
+      <c r="B76" s="18"/>
+      <c r="C76" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D76" s="6" t="s">
+      <c r="D76" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E76" s="9"/>
-    </row>
-    <row r="77" spans="1:5" ht="15.75">
-      <c r="A77" s="8">
+      <c r="E76" s="6"/>
+    </row>
+    <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A77" s="18">
         <v>9</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="B77" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="C77" s="6" t="s">
+      <c r="C77" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D77" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E77" s="9"/>
-    </row>
-    <row r="78" spans="1:5" ht="15.75">
-      <c r="A78" s="8"/>
-      <c r="B78" s="8"/>
-      <c r="C78" s="6" t="s">
+      <c r="D77" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E77" s="6"/>
+    </row>
+    <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A78" s="18"/>
+      <c r="B78" s="18"/>
+      <c r="C78" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D78" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E78" s="9"/>
-    </row>
-    <row r="79" spans="1:5" ht="15.75">
-      <c r="A79" s="8"/>
-      <c r="B79" s="8"/>
-      <c r="C79" s="6" t="s">
+      <c r="D78" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E78" s="6"/>
+    </row>
+    <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A79" s="18"/>
+      <c r="B79" s="18"/>
+      <c r="C79" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D79" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E79" s="9"/>
-    </row>
-    <row r="80" spans="1:5" ht="15.75">
-      <c r="A80" s="8">
+      <c r="D79" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E79" s="6"/>
+    </row>
+    <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A80" s="18">
         <v>10</v>
       </c>
-      <c r="B80" s="8" t="s">
+      <c r="B80" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="C80" s="6" t="s">
+      <c r="C80" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D80" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E80" s="9"/>
-    </row>
-    <row r="81" spans="1:5" ht="15.75">
-      <c r="A81" s="8"/>
-      <c r="B81" s="8"/>
-      <c r="C81" s="6" t="s">
+      <c r="D80" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E80" s="6"/>
+    </row>
+    <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A81" s="18"/>
+      <c r="B81" s="18"/>
+      <c r="C81" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D81" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E81" s="9"/>
-    </row>
-    <row r="82" spans="1:5" ht="15.75">
-      <c r="A82" s="8"/>
-      <c r="B82" s="8"/>
-      <c r="C82" s="6" t="s">
+      <c r="D81" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E81" s="6"/>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A82" s="18"/>
+      <c r="B82" s="18"/>
+      <c r="C82" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D82" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E82" s="9"/>
-    </row>
-    <row r="83" spans="1:5" ht="15.75">
-      <c r="A83" s="8"/>
-      <c r="B83" s="8"/>
-      <c r="C83" s="6" t="s">
+      <c r="D82" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E82" s="6"/>
+    </row>
+    <row r="83" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A83" s="18"/>
+      <c r="B83" s="18"/>
+      <c r="C83" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D83" s="6" t="s">
+      <c r="D83" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E83" s="9"/>
-    </row>
-    <row r="84" spans="1:5" ht="15.75">
-      <c r="A84" s="8"/>
-      <c r="B84" s="8"/>
-      <c r="C84" s="6" t="s">
+      <c r="E83" s="6"/>
+    </row>
+    <row r="84" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A84" s="18"/>
+      <c r="B84" s="18"/>
+      <c r="C84" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D84" s="6" t="s">
+      <c r="D84" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E84" s="9"/>
-    </row>
-    <row r="85" spans="1:5" ht="15.75">
-      <c r="A85" s="8">
+      <c r="E84" s="6"/>
+    </row>
+    <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A85" s="18">
         <v>11</v>
       </c>
-      <c r="B85" s="8" t="s">
+      <c r="B85" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="C85" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D85" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E85" s="9"/>
-    </row>
-    <row r="86" spans="1:5" ht="15.75">
-      <c r="A86" s="8"/>
-      <c r="B86" s="8"/>
-      <c r="C86" s="6" t="s">
+      <c r="D85" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E85" s="6"/>
+    </row>
+    <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A86" s="18"/>
+      <c r="B86" s="18"/>
+      <c r="C86" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D86" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E86" s="9"/>
-    </row>
-    <row r="87" spans="1:5" ht="15.75">
-      <c r="A87" s="8"/>
-      <c r="B87" s="8"/>
-      <c r="C87" s="6" t="s">
+      <c r="D86" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E86" s="6"/>
+    </row>
+    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A87" s="18"/>
+      <c r="B87" s="18"/>
+      <c r="C87" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D87" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E87" s="9"/>
-    </row>
-    <row r="88" spans="1:5" ht="15.75">
-      <c r="A88" s="8"/>
-      <c r="B88" s="8"/>
-      <c r="C88" s="6" t="s">
+      <c r="D87" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E87" s="6"/>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A88" s="18"/>
+      <c r="B88" s="18"/>
+      <c r="C88" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D88" s="6" t="s">
+      <c r="D88" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E88" s="9"/>
-    </row>
-    <row r="89" spans="1:5" ht="15.75">
-      <c r="A89" s="8">
+      <c r="E88" s="6"/>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A89" s="18">
         <v>12</v>
       </c>
-      <c r="B89" s="8" t="s">
+      <c r="B89" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C89" s="6" t="s">
+      <c r="C89" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D89" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E89" s="10" t="s">
+      <c r="D89" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E89" s="19" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15.75">
-      <c r="A90" s="8"/>
-      <c r="B90" s="8"/>
-      <c r="C90" s="6" t="s">
+    <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A90" s="18"/>
+      <c r="B90" s="18"/>
+      <c r="C90" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D90" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E90" s="11"/>
-    </row>
-    <row r="91" spans="1:5" ht="15.75">
-      <c r="A91" s="8"/>
-      <c r="B91" s="8"/>
-      <c r="C91" s="6" t="s">
+      <c r="D90" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E90" s="16"/>
+    </row>
+    <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A91" s="18"/>
+      <c r="B91" s="18"/>
+      <c r="C91" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D91" s="6" t="s">
+      <c r="D91" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E91" s="12"/>
-    </row>
-    <row r="92" spans="1:5" ht="15.75">
-      <c r="A92" s="8">
+      <c r="E91" s="17"/>
+    </row>
+    <row r="92" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A92" s="18">
         <v>13</v>
       </c>
-      <c r="B92" s="8" t="s">
+      <c r="B92" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C92" s="6" t="s">
+      <c r="C92" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D92" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E92" s="13" t="s">
+      <c r="D92" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E92" s="15" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="15.75">
-      <c r="A93" s="8"/>
-      <c r="B93" s="8"/>
-      <c r="C93" s="6" t="s">
+    <row r="93" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A93" s="18"/>
+      <c r="B93" s="18"/>
+      <c r="C93" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D93" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E93" s="11"/>
-    </row>
-    <row r="94" spans="1:5" ht="15.75">
-      <c r="A94" s="8"/>
-      <c r="B94" s="8"/>
-      <c r="C94" s="6" t="s">
+      <c r="D93" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E93" s="16"/>
+    </row>
+    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A94" s="18"/>
+      <c r="B94" s="18"/>
+      <c r="C94" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D94" s="6" t="s">
+      <c r="D94" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E94" s="11"/>
-    </row>
-    <row r="95" spans="1:5" ht="15.75">
-      <c r="A95" s="8"/>
-      <c r="B95" s="8"/>
-      <c r="C95" s="6" t="s">
+      <c r="E94" s="16"/>
+    </row>
+    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A95" s="18"/>
+      <c r="B95" s="18"/>
+      <c r="C95" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D95" s="6" t="s">
+      <c r="D95" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E95" s="11"/>
-    </row>
-    <row r="96" spans="1:5" ht="15.75">
-      <c r="A96" s="8"/>
-      <c r="B96" s="8"/>
-      <c r="C96" s="6" t="s">
+      <c r="E95" s="16"/>
+    </row>
+    <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A96" s="18"/>
+      <c r="B96" s="18"/>
+      <c r="C96" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D96" s="6" t="s">
+      <c r="D96" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E96" s="11"/>
-    </row>
-    <row r="97" spans="1:5" ht="15.75">
-      <c r="A97" s="8"/>
-      <c r="B97" s="8"/>
-      <c r="C97" s="6" t="s">
+      <c r="E96" s="16"/>
+    </row>
+    <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A97" s="18"/>
+      <c r="B97" s="18"/>
+      <c r="C97" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D97" s="6" t="s">
+      <c r="D97" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E97" s="11"/>
-    </row>
-    <row r="98" spans="1:5" ht="15.75">
-      <c r="A98" s="8"/>
-      <c r="B98" s="8"/>
-      <c r="C98" s="6" t="s">
+      <c r="E97" s="16"/>
+    </row>
+    <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A98" s="18"/>
+      <c r="B98" s="18"/>
+      <c r="C98" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D98" s="6" t="s">
+      <c r="D98" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E98" s="11"/>
-    </row>
-    <row r="99" spans="1:5" ht="15.75">
-      <c r="A99" s="8"/>
-      <c r="B99" s="8"/>
-      <c r="C99" s="6" t="s">
+      <c r="E98" s="16"/>
+    </row>
+    <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A99" s="18"/>
+      <c r="B99" s="18"/>
+      <c r="C99" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D99" s="6" t="s">
+      <c r="D99" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E99" s="12"/>
-    </row>
-    <row r="100" spans="1:5" ht="15.75">
-      <c r="A100" s="8">
+      <c r="E99" s="16"/>
+    </row>
+    <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A100" s="18"/>
+      <c r="B100" s="18"/>
+      <c r="C100" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E100" s="16"/>
+    </row>
+    <row r="101" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A101" s="18"/>
+      <c r="B101" s="18"/>
+      <c r="C101" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="D101" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E101" s="17"/>
+    </row>
+    <row r="102" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A102" s="18">
         <v>14</v>
       </c>
-      <c r="B100" s="8" t="s">
+      <c r="B102" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="C100" s="6" t="s">
+      <c r="C102" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D100" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E100" s="14" t="s">
+      <c r="D102" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E102" s="12" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15.75">
-      <c r="A101" s="8"/>
-      <c r="B101" s="8"/>
-      <c r="C101" s="6" t="s">
+    <row r="103" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A103" s="18"/>
+      <c r="B103" s="18"/>
+      <c r="C103" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D101" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E101" s="15"/>
-    </row>
-    <row r="102" spans="1:5" ht="15.75">
-      <c r="A102" s="8"/>
-      <c r="B102" s="8"/>
-      <c r="C102" s="6" t="s">
+      <c r="D103" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E103" s="13"/>
+    </row>
+    <row r="104" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A104" s="18"/>
+      <c r="B104" s="18"/>
+      <c r="C104" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D102" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E102" s="15"/>
-    </row>
-    <row r="103" spans="1:5" ht="15.75">
-      <c r="A103" s="8"/>
-      <c r="B103" s="8"/>
-      <c r="C103" s="6" t="s">
+      <c r="D104" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E104" s="13"/>
+    </row>
+    <row r="105" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A105" s="18"/>
+      <c r="B105" s="18"/>
+      <c r="C105" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D103" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E103" s="16"/>
-    </row>
-    <row r="104" spans="1:5" ht="15.75">
-      <c r="A104" s="8">
+      <c r="D105" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E105" s="14"/>
+    </row>
+    <row r="106" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A106" s="18">
         <v>15</v>
       </c>
-      <c r="B104" s="8" t="s">
+      <c r="B106" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="C104" s="6" t="s">
+      <c r="C106" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D104" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E104" s="13" t="s">
+      <c r="D106" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E106" s="15" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="15.75">
-      <c r="A105" s="8"/>
-      <c r="B105" s="8"/>
-      <c r="C105" s="6" t="s">
+    <row r="107" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A107" s="18"/>
+      <c r="B107" s="18"/>
+      <c r="C107" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D105" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E105" s="11"/>
-    </row>
-    <row r="106" spans="1:5" ht="15.75">
-      <c r="A106" s="8"/>
-      <c r="B106" s="8"/>
-      <c r="C106" s="6" t="s">
+      <c r="D107" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E107" s="16"/>
+    </row>
+    <row r="108" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A108" s="18"/>
+      <c r="B108" s="18"/>
+      <c r="C108" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D106" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E106" s="11"/>
-    </row>
-    <row r="107" spans="1:5" ht="15.75">
-      <c r="A107" s="8"/>
-      <c r="B107" s="8"/>
-      <c r="C107" s="6" t="s">
+      <c r="D108" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E108" s="16"/>
+    </row>
+    <row r="109" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A109" s="18"/>
+      <c r="B109" s="18"/>
+      <c r="C109" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D107" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E107" s="12"/>
-    </row>
-    <row r="108" spans="1:5" ht="15.75">
-      <c r="A108" s="8">
-        <v>16</v>
-      </c>
-      <c r="B108" s="8" t="s">
+      <c r="D109" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E109" s="17"/>
+    </row>
+    <row r="110" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A110" s="18">
+        <v>16</v>
+      </c>
+      <c r="B110" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="C108" s="6" t="s">
+      <c r="C110" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D108" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E108" s="9"/>
-    </row>
-    <row r="109" spans="1:5" ht="15.75">
-      <c r="A109" s="8"/>
-      <c r="B109" s="8"/>
-      <c r="C109" s="6" t="s">
+      <c r="D110" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E110" s="6"/>
+    </row>
+    <row r="111" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A111" s="18"/>
+      <c r="B111" s="18"/>
+      <c r="C111" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D109" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E109" s="9"/>
-    </row>
-    <row r="110" spans="1:5" ht="15.75">
-      <c r="A110" s="8"/>
-      <c r="B110" s="8"/>
-      <c r="C110" s="6" t="s">
+      <c r="D111" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E111" s="6"/>
+    </row>
+    <row r="112" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A112" s="18"/>
+      <c r="B112" s="18"/>
+      <c r="C112" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D110" s="6" t="s">
+      <c r="D112" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E110" s="9"/>
-    </row>
-    <row r="111" spans="1:5" ht="15.75">
-      <c r="A111" s="8"/>
-      <c r="B111" s="8"/>
-      <c r="C111" s="6" t="s">
+      <c r="E112" s="6"/>
+    </row>
+    <row r="113" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A113" s="18"/>
+      <c r="B113" s="18"/>
+      <c r="C113" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D111" s="6" t="s">
+      <c r="D113" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E111" s="9"/>
-    </row>
-    <row r="112" spans="1:5" ht="15.75">
-      <c r="A112" s="8"/>
-      <c r="B112" s="8"/>
-      <c r="C112" s="6" t="s">
+      <c r="E113" s="6"/>
+    </row>
+    <row r="114" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A114" s="18"/>
+      <c r="B114" s="18"/>
+      <c r="C114" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D112" s="6" t="s">
+      <c r="D114" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E112" s="9"/>
-    </row>
-    <row r="113" spans="1:5" ht="15.75">
-      <c r="A113" s="8"/>
-      <c r="B113" s="8"/>
-      <c r="C113" s="6" t="s">
+      <c r="E114" s="6"/>
+    </row>
+    <row r="115" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A115" s="18"/>
+      <c r="B115" s="18"/>
+      <c r="C115" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D113" s="6" t="s">
+      <c r="D115" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E113" s="9"/>
-    </row>
-    <row r="114" spans="1:5" ht="15.75">
-      <c r="A114" s="8"/>
-      <c r="B114" s="8"/>
-      <c r="C114" s="6" t="s">
+      <c r="E115" s="6"/>
+    </row>
+    <row r="116" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A116" s="18"/>
+      <c r="B116" s="18"/>
+      <c r="C116" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D114" s="6" t="s">
+      <c r="D116" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E114" s="9"/>
-    </row>
-    <row r="115" spans="1:5" ht="15.75">
-      <c r="A115" s="8"/>
-      <c r="B115" s="8"/>
-      <c r="C115" s="6" t="s">
+      <c r="E116" s="6"/>
+    </row>
+    <row r="117" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A117" s="18"/>
+      <c r="B117" s="18"/>
+      <c r="C117" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D115" s="6" t="s">
+      <c r="D117" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E115" s="9"/>
-    </row>
-    <row r="116" spans="1:5" ht="15.75">
-      <c r="A116" s="8"/>
-      <c r="B116" s="8"/>
-      <c r="C116" s="6" t="s">
+      <c r="E117" s="6"/>
+    </row>
+    <row r="118" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A118" s="18"/>
+      <c r="B118" s="18"/>
+      <c r="C118" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D116" s="6" t="s">
+      <c r="D118" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E116" s="9"/>
-    </row>
-    <row r="117" spans="1:5" ht="15.75">
-      <c r="A117" s="8"/>
-      <c r="B117" s="8"/>
-      <c r="C117" s="6" t="s">
+      <c r="E118" s="6"/>
+    </row>
+    <row r="119" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A119" s="18"/>
+      <c r="B119" s="18"/>
+      <c r="C119" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D117" s="6" t="s">
+      <c r="D119" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E117" s="9"/>
-    </row>
-    <row r="118" spans="1:5" ht="15.75">
-      <c r="A118" s="8"/>
-      <c r="B118" s="8"/>
-      <c r="C118" s="6" t="s">
+      <c r="E119" s="6"/>
+    </row>
+    <row r="120" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A120" s="18"/>
+      <c r="B120" s="18"/>
+      <c r="C120" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D118" s="6" t="s">
+      <c r="D120" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E118" s="9"/>
-    </row>
-    <row r="119" spans="1:5" ht="15.75">
-      <c r="A119" s="8"/>
-      <c r="B119" s="8"/>
-      <c r="C119" s="6" t="s">
+      <c r="E120" s="6"/>
+    </row>
+    <row r="121" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A121" s="18"/>
+      <c r="B121" s="18"/>
+      <c r="C121" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D119" s="6" t="s">
+      <c r="D121" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E119" s="9"/>
-    </row>
-    <row r="120" spans="1:5" ht="15.75">
-      <c r="A120" s="8">
+      <c r="E121" s="6"/>
+    </row>
+    <row r="122" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A122" s="18">
         <v>17</v>
       </c>
-      <c r="B120" s="8" t="s">
+      <c r="B122" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="C120" s="6" t="s">
+      <c r="C122" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D120" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E120" s="9"/>
-    </row>
-    <row r="121" spans="1:5" ht="15.75">
-      <c r="A121" s="8"/>
-      <c r="B121" s="8"/>
-      <c r="C121" s="6" t="s">
+      <c r="D122" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E122" s="6"/>
+    </row>
+    <row r="123" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A123" s="18"/>
+      <c r="B123" s="18"/>
+      <c r="C123" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D121" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E121" s="9"/>
-    </row>
-    <row r="122" spans="1:5" ht="15.75">
-      <c r="A122" s="8"/>
-      <c r="B122" s="8"/>
-      <c r="C122" s="6" t="s">
+      <c r="D123" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E123" s="6"/>
+    </row>
+    <row r="124" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A124" s="18"/>
+      <c r="B124" s="18"/>
+      <c r="C124" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D122" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E122" s="9"/>
-    </row>
-    <row r="123" spans="1:5" ht="15.75">
-      <c r="A123" s="8"/>
-      <c r="B123" s="8"/>
-      <c r="C123" s="6" t="s">
+      <c r="D124" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E124" s="6"/>
+    </row>
+    <row r="125" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A125" s="18"/>
+      <c r="B125" s="18"/>
+      <c r="C125" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D123" s="6" t="s">
+      <c r="D125" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E123" s="9"/>
-    </row>
-    <row r="124" spans="1:5" ht="15.75">
-      <c r="A124" s="8"/>
-      <c r="B124" s="8"/>
-      <c r="C124" s="6" t="s">
+      <c r="E125" s="6"/>
+    </row>
+    <row r="126" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A126" s="18"/>
+      <c r="B126" s="18"/>
+      <c r="C126" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D124" s="6" t="s">
+      <c r="D126" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E124" s="9"/>
-    </row>
-    <row r="125" spans="1:5" ht="15.75">
-      <c r="A125" s="8"/>
-      <c r="B125" s="8"/>
-      <c r="C125" s="6" t="s">
+      <c r="E126" s="6"/>
+    </row>
+    <row r="127" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A127" s="18"/>
+      <c r="B127" s="18"/>
+      <c r="C127" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D125" s="6" t="s">
+      <c r="D127" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E125" s="9"/>
-    </row>
-    <row r="126" spans="1:5" ht="15.75">
-      <c r="A126" s="8"/>
-      <c r="B126" s="8"/>
-      <c r="C126" s="6" t="s">
+      <c r="E127" s="6"/>
+    </row>
+    <row r="128" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A128" s="18"/>
+      <c r="B128" s="18"/>
+      <c r="C128" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D126" s="6" t="s">
+      <c r="D128" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E126" s="9"/>
-    </row>
-    <row r="127" spans="1:5" ht="15.75">
-      <c r="A127" s="8"/>
-      <c r="B127" s="8"/>
-      <c r="C127" s="6" t="s">
+      <c r="E128" s="6"/>
+    </row>
+    <row r="129" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A129" s="18"/>
+      <c r="B129" s="18"/>
+      <c r="C129" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D127" s="6" t="s">
+      <c r="D129" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E127" s="9"/>
-    </row>
-    <row r="128" spans="1:5" ht="15.75">
-      <c r="A128" s="8"/>
-      <c r="B128" s="8"/>
-      <c r="C128" s="6" t="s">
+      <c r="E129" s="6"/>
+    </row>
+    <row r="130" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A130" s="18"/>
+      <c r="B130" s="18"/>
+      <c r="C130" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D128" s="6" t="s">
+      <c r="D130" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E128" s="9"/>
-    </row>
-    <row r="129" spans="1:5" ht="15.75">
-      <c r="A129" s="8"/>
-      <c r="B129" s="8"/>
-      <c r="C129" s="6" t="s">
+      <c r="E130" s="6"/>
+    </row>
+    <row r="131" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A131" s="18"/>
+      <c r="B131" s="18"/>
+      <c r="C131" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D129" s="6" t="s">
+      <c r="D131" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E129" s="9"/>
-    </row>
-    <row r="130" spans="1:5" ht="15.75">
-      <c r="A130" s="8"/>
-      <c r="B130" s="8"/>
-      <c r="C130" s="6" t="s">
+      <c r="E131" s="6"/>
+    </row>
+    <row r="132" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A132" s="18"/>
+      <c r="B132" s="18"/>
+      <c r="C132" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D130" s="6" t="s">
+      <c r="D132" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E130" s="9"/>
-    </row>
-    <row r="131" spans="1:5" ht="15.75">
-      <c r="A131" s="8"/>
-      <c r="B131" s="8"/>
-      <c r="C131" s="6" t="s">
+      <c r="E132" s="6"/>
+    </row>
+    <row r="133" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A133" s="18"/>
+      <c r="B133" s="18"/>
+      <c r="C133" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D131" s="6" t="s">
+      <c r="D133" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E131" s="9"/>
-    </row>
-    <row r="132" spans="1:5" ht="15.75">
-      <c r="A132" s="8"/>
-      <c r="B132" s="8"/>
-      <c r="C132" s="6" t="s">
+      <c r="E133" s="6"/>
+    </row>
+    <row r="134" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A134" s="18"/>
+      <c r="B134" s="18"/>
+      <c r="C134" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D132" s="6" t="s">
+      <c r="D134" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E132" s="9"/>
-    </row>
-    <row r="133" spans="1:5" ht="15.75">
-      <c r="A133" s="8"/>
-      <c r="B133" s="8"/>
-      <c r="C133" s="6" t="s">
+      <c r="E134" s="6"/>
+    </row>
+    <row r="135" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A135" s="18"/>
+      <c r="B135" s="18"/>
+      <c r="C135" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D133" s="6" t="s">
+      <c r="D135" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E133" s="9"/>
-    </row>
-    <row r="134" spans="1:5" ht="15.75">
-      <c r="A134" s="8"/>
-      <c r="B134" s="8"/>
-      <c r="C134" s="6" t="s">
+      <c r="E135" s="6"/>
+    </row>
+    <row r="136" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A136" s="18"/>
+      <c r="B136" s="18"/>
+      <c r="C136" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D134" s="6" t="s">
+      <c r="D136" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E134" s="9"/>
+      <c r="E136" s="6"/>
+    </row>
+    <row r="137" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A137" s="20">
+        <v>18</v>
+      </c>
+      <c r="B137" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="C137" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D137" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E137" s="2"/>
+    </row>
+    <row r="138" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A138" s="20"/>
+      <c r="B138" s="20"/>
+      <c r="C138" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="D138" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E138" s="2"/>
+    </row>
+    <row r="139" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A139" s="20"/>
+      <c r="B139" s="20"/>
+      <c r="C139" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D139" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E139" s="2"/>
+    </row>
+    <row r="140" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A140" s="20"/>
+      <c r="B140" s="20"/>
+      <c r="C140" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D140" s="24" t="s">
+        <v>223</v>
+      </c>
+      <c r="E140" s="2"/>
+    </row>
+    <row r="141" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A141" s="20"/>
+      <c r="B141" s="20"/>
+      <c r="C141" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="D141" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A142" s="20"/>
+      <c r="B142" s="20"/>
+      <c r="C142" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E142" s="2"/>
+    </row>
+    <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A143" s="20"/>
+      <c r="B143" s="20"/>
+      <c r="C143" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D143" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E143" s="2"/>
+    </row>
+    <row r="144" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A144" s="20"/>
+      <c r="B144" s="20"/>
+      <c r="C144" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D144" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E144" s="2"/>
+    </row>
+    <row r="145" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A145" s="20"/>
+      <c r="B145" s="20"/>
+      <c r="C145" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D145" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E145" s="2"/>
+    </row>
+    <row r="146" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A146" s="20"/>
+      <c r="B146" s="20"/>
+      <c r="C146" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D146" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E146" s="2"/>
+    </row>
+    <row r="147" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A147" s="20"/>
+      <c r="B147" s="20"/>
+      <c r="C147" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D147" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E147" s="2"/>
+    </row>
+    <row r="148" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A148" s="20">
+        <v>19</v>
+      </c>
+      <c r="B148" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="C148" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D148" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E148" s="2"/>
+    </row>
+    <row r="149" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A149" s="20"/>
+      <c r="B149" s="20"/>
+      <c r="C149" s="24" t="s">
+        <v>225</v>
+      </c>
+      <c r="D149" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E149" s="2"/>
+    </row>
+    <row r="150" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A150" s="20"/>
+      <c r="B150" s="20"/>
+      <c r="C150" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="D150" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A151" s="20"/>
+      <c r="B151" s="20"/>
+      <c r="C151" s="24" t="s">
+        <v>227</v>
+      </c>
+      <c r="D151" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A152" s="20"/>
+      <c r="B152" s="20"/>
+      <c r="C152" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D152" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>233</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="E100:E103"/>
-    <mergeCell ref="E104:E107"/>
-    <mergeCell ref="A28:A32"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="A17:A23"/>
+  <mergeCells count="42">
+    <mergeCell ref="B137:B147"/>
+    <mergeCell ref="B148:B152"/>
+    <mergeCell ref="A137:A147"/>
+    <mergeCell ref="A148:A152"/>
+    <mergeCell ref="B7:B16"/>
+    <mergeCell ref="B17:B23"/>
+    <mergeCell ref="B28:B32"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="B122:B136"/>
+    <mergeCell ref="A122:A136"/>
+    <mergeCell ref="A110:A121"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="B110:B121"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="B102:B105"/>
     <mergeCell ref="A7:A16"/>
     <mergeCell ref="E89:E91"/>
-    <mergeCell ref="E92:E99"/>
+    <mergeCell ref="E92:E101"/>
     <mergeCell ref="A80:A84"/>
     <mergeCell ref="A77:A79"/>
     <mergeCell ref="A66:A76"/>
@@ -3142,29 +3508,21 @@
     <mergeCell ref="A36:A50"/>
     <mergeCell ref="A33:A35"/>
     <mergeCell ref="B85:B88"/>
-    <mergeCell ref="B120:B134"/>
-    <mergeCell ref="A120:A134"/>
-    <mergeCell ref="A108:A119"/>
-    <mergeCell ref="A104:A107"/>
-    <mergeCell ref="A100:A103"/>
-    <mergeCell ref="A92:A99"/>
+    <mergeCell ref="A92:A101"/>
     <mergeCell ref="A89:A91"/>
     <mergeCell ref="A85:A88"/>
     <mergeCell ref="B36:B50"/>
     <mergeCell ref="B51:B65"/>
     <mergeCell ref="B66:B76"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="A28:A32"/>
+    <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A17:A23"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="B80:B84"/>
-    <mergeCell ref="B108:B119"/>
-    <mergeCell ref="B104:B107"/>
-    <mergeCell ref="B100:B103"/>
-    <mergeCell ref="B92:B99"/>
+    <mergeCell ref="B92:B101"/>
     <mergeCell ref="B89:B91"/>
-    <mergeCell ref="B7:B16"/>
-    <mergeCell ref="B17:B23"/>
-    <mergeCell ref="B28:B32"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B33:B35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3174,15 +3532,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D659272-F48A-4C07-A3BF-4D5B739EFB06}">
-  <dimension ref="B3:K40"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="B3:K50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="5.42578125" customWidth="1"/>
     <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" customWidth="1"/>
-    <col min="6" max="6" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="42.5703125" customWidth="1"/>
+    <col min="6" max="6" width="36.140625" customWidth="1"/>
     <col min="7" max="7" width="42" customWidth="1"/>
     <col min="8" max="8" width="61.28515625" customWidth="1"/>
     <col min="9" max="9" width="62.140625" hidden="1" customWidth="1"/>
@@ -3190,17 +3548,17 @@
     <col min="11" max="11" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="F3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="19.5">
+    <row r="4" spans="2:11" ht="19.5" x14ac:dyDescent="0.3">
       <c r="D4" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="2:11">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>97</v>
       </c>
@@ -3219,7 +3577,7 @@
       <c r="G6" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="2" t="s">
         <v>116</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -3232,14 +3590,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:11">
-      <c r="B7" s="3" t="s">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>1</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -3262,12 +3620,12 @@
       </c>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="2:11">
-      <c r="B8" s="3"/>
-      <c r="C8" s="5">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="20"/>
+      <c r="C8" s="3">
         <v>2</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -3290,12 +3648,12 @@
       </c>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="2:11">
-      <c r="B9" s="3"/>
-      <c r="C9" s="5">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="20"/>
+      <c r="C9" s="3">
         <v>3</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -3318,12 +3676,12 @@
       </c>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="2:11">
-      <c r="B10" s="3"/>
-      <c r="C10" s="5">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="20"/>
+      <c r="C10" s="3">
         <v>4</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -3346,12 +3704,12 @@
       </c>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="2:11">
-      <c r="B11" s="3"/>
-      <c r="C11" s="5">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="20"/>
+      <c r="C11" s="3">
         <v>5</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -3374,14 +3732,14 @@
       </c>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="2:11">
-      <c r="B12" s="3" t="s">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <v>6</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -3404,12 +3762,12 @@
       </c>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="2:11">
-      <c r="B13" s="3"/>
-      <c r="C13" s="5">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="20"/>
+      <c r="C13" s="3">
         <v>7</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E13" s="2" t="s">
@@ -3432,12 +3790,12 @@
       </c>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="2:11">
-      <c r="B14" s="3"/>
-      <c r="C14" s="5">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="20"/>
+      <c r="C14" s="3">
         <v>8</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -3460,12 +3818,12 @@
       </c>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="2:11">
-      <c r="B15" s="3"/>
-      <c r="C15" s="5">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B15" s="20"/>
+      <c r="C15" s="3">
         <v>9</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -3488,12 +3846,12 @@
       </c>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="2:11">
-      <c r="B16" s="3"/>
-      <c r="C16" s="5">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="20"/>
+      <c r="C16" s="3">
         <v>10</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -3516,14 +3874,14 @@
       </c>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="2:11">
-      <c r="B17" s="3" t="s">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="3">
         <v>11</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E17" s="2" t="s">
@@ -3541,17 +3899,17 @@
       <c r="I17" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="21" t="s">
         <v>167</v>
       </c>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="2:11">
-      <c r="B18" s="3"/>
-      <c r="C18" s="5">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B18" s="20"/>
+      <c r="C18" s="3">
         <v>12</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E18" s="2" t="s">
@@ -3569,15 +3927,15 @@
       <c r="I18" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="J18" s="4"/>
+      <c r="J18" s="22"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="2:11">
-      <c r="B19" s="3"/>
-      <c r="C19" s="5">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B19" s="20"/>
+      <c r="C19" s="3">
         <v>13</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E19" s="2" t="s">
@@ -3595,15 +3953,15 @@
       <c r="I19" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="J19" s="4"/>
+      <c r="J19" s="22"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="2:11">
-      <c r="B20" s="3"/>
-      <c r="C20" s="5">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B20" s="20"/>
+      <c r="C20" s="3">
         <v>14</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E20" s="2" t="s">
@@ -3621,15 +3979,15 @@
       <c r="I20" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="J20" s="4"/>
+      <c r="J20" s="22"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="2:11">
-      <c r="B21" s="3"/>
-      <c r="C21" s="5">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B21" s="20"/>
+      <c r="C21" s="3">
         <v>15</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E21" s="2" t="s">
@@ -3647,17 +4005,17 @@
       <c r="I21" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="J21" s="4"/>
+      <c r="J21" s="22"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="2:11">
-      <c r="B22" s="3" t="s">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B22" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="C22" s="5">
-        <v>16</v>
-      </c>
-      <c r="D22" s="5" t="s">
+      <c r="C22" s="3">
+        <v>16</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E22" s="2" t="s">
@@ -3676,12 +4034,12 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="2:11">
-      <c r="B23" s="3"/>
-      <c r="C23" s="5">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B23" s="20"/>
+      <c r="C23" s="3">
         <v>17</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E23" s="2" t="s">
@@ -3700,12 +4058,12 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="2:11">
-      <c r="B24" s="3"/>
-      <c r="C24" s="5">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B24" s="20"/>
+      <c r="C24" s="3">
         <v>18</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E24" s="2" t="s">
@@ -3724,12 +4082,12 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="2:11">
-      <c r="B25" s="3"/>
-      <c r="C25" s="5">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B25" s="20"/>
+      <c r="C25" s="3">
         <v>19</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E25" s="2" t="s">
@@ -3748,12 +4106,12 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="2:11">
-      <c r="B26" s="3"/>
-      <c r="C26" s="5">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B26" s="20"/>
+      <c r="C26" s="3">
         <v>20</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E26" s="2" t="s">
@@ -3772,12 +4130,12 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="2:11">
-      <c r="B27" s="3"/>
-      <c r="C27" s="5">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B27" s="20"/>
+      <c r="C27" s="3">
         <v>21</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E27" s="2" t="s">
@@ -3796,14 +4154,14 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="2:11">
-      <c r="B28" s="3" t="s">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B28" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="3">
         <v>22</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E28" s="2" t="s">
@@ -3822,12 +4180,12 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="2:11">
-      <c r="B29" s="3"/>
-      <c r="C29" s="5">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B29" s="20"/>
+      <c r="C29" s="3">
         <v>23</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E29" s="2" t="s">
@@ -3846,12 +4204,12 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="2:11">
-      <c r="B30" s="3"/>
-      <c r="C30" s="5">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B30" s="20"/>
+      <c r="C30" s="3">
         <v>24</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E30" s="2" t="s">
@@ -3870,12 +4228,12 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="2:11">
-      <c r="B31" s="3"/>
-      <c r="C31" s="5">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B31" s="20"/>
+      <c r="C31" s="3">
         <v>25</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E31" s="2" t="s">
@@ -3894,12 +4252,12 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="2:11">
-      <c r="B32" s="3"/>
-      <c r="C32" s="5">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B32" s="20"/>
+      <c r="C32" s="3">
         <v>26</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E32" s="2" t="s">
@@ -3918,12 +4276,12 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="2:11">
-      <c r="B33" s="3"/>
-      <c r="C33" s="5">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B33" s="20"/>
+      <c r="C33" s="3">
         <v>27</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E33" s="2" t="s">
@@ -3942,14 +4300,14 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="2:11">
-      <c r="B34" s="3" t="s">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B34" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C34" s="3">
         <v>28</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E34" s="2" t="s">
@@ -3968,12 +4326,12 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="2:11">
-      <c r="B35" s="3"/>
-      <c r="C35" s="5">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B35" s="20"/>
+      <c r="C35" s="3">
         <v>29</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E35" s="2" t="s">
@@ -3992,12 +4350,12 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
     </row>
-    <row r="36" spans="2:11">
-      <c r="B36" s="3"/>
-      <c r="C36" s="5">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B36" s="20"/>
+      <c r="C36" s="3">
         <v>30</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E36" s="2" t="s">
@@ -4016,12 +4374,12 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="2:11">
-      <c r="B37" s="3"/>
-      <c r="C37" s="5">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B37" s="20"/>
+      <c r="C37" s="3">
         <v>31</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E37" s="2" t="s">
@@ -4040,12 +4398,12 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
     </row>
-    <row r="38" spans="2:11">
-      <c r="B38" s="3"/>
-      <c r="C38" s="5">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B38" s="20"/>
+      <c r="C38" s="3">
         <v>32</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E38" s="2" t="s">
@@ -4064,12 +4422,12 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
     </row>
-    <row r="39" spans="2:11">
-      <c r="B39" s="3"/>
-      <c r="C39" s="5">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B39" s="20"/>
+      <c r="C39" s="3">
         <v>33</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E39" s="2" t="s">
@@ -4088,12 +4446,12 @@
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
     </row>
-    <row r="40" spans="2:11">
-      <c r="B40" s="3"/>
-      <c r="C40" s="5">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B40" s="20"/>
+      <c r="C40" s="3">
         <v>34</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E40" s="2" t="s">
@@ -4112,8 +4470,242 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
     </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B41" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="C41" s="3">
+        <v>35</v>
+      </c>
+      <c r="D41" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E41" s="26" t="s">
+        <v>235</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+    </row>
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B42" s="20"/>
+      <c r="C42" s="3">
+        <v>36</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E42" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B43" s="20"/>
+      <c r="C43" s="3">
+        <v>37</v>
+      </c>
+      <c r="D43" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E43" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+    </row>
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B44" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="C44" s="3">
+        <v>38</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E44" s="26" t="s">
+        <v>238</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+    </row>
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B45" s="20"/>
+      <c r="C45" s="3">
+        <v>39</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E45" s="26" t="s">
+        <v>239</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+    </row>
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B46" s="20"/>
+      <c r="C46" s="3">
+        <v>40</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E46" s="26" t="s">
+        <v>240</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+    </row>
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B47" s="20"/>
+      <c r="C47" s="3">
+        <v>41</v>
+      </c>
+      <c r="D47" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E47" s="26" t="s">
+        <v>241</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+    </row>
+    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B48" s="20"/>
+      <c r="C48" s="3">
+        <v>42</v>
+      </c>
+      <c r="D48" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="E48" s="26" t="s">
+        <v>242</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+    </row>
+    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B49" s="20"/>
+      <c r="C49" s="27">
+        <v>43</v>
+      </c>
+      <c r="D49" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="E49" s="29"/>
+      <c r="F49" s="29" t="s">
+        <v>252</v>
+      </c>
+      <c r="G49" s="29"/>
+      <c r="H49" s="29"/>
+      <c r="I49" s="29"/>
+      <c r="J49" s="29"/>
+      <c r="K49" s="29"/>
+    </row>
+    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B50" s="20"/>
+      <c r="C50" s="27">
+        <v>44</v>
+      </c>
+      <c r="D50" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="E50" s="29"/>
+      <c r="F50" s="29" t="s">
+        <v>251</v>
+      </c>
+      <c r="G50" s="29"/>
+      <c r="H50" s="29"/>
+      <c r="I50" s="29"/>
+      <c r="J50" s="29"/>
+      <c r="K50" s="29"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B44:B50"/>
     <mergeCell ref="B7:B11"/>
     <mergeCell ref="B34:B40"/>
     <mergeCell ref="J17:J21"/>
@@ -4129,259 +4721,259 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB413690-E0CE-4831-9E46-1DB31698C173}">
   <dimension ref="W25:AP48"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="25" spans="23:33" ht="22.5">
-      <c r="W25" s="18" t="s">
+    <row r="25" spans="23:33" ht="22.5" x14ac:dyDescent="0.35">
+      <c r="W25" s="7" t="s">
         <v>212</v>
       </c>
       <c r="Y25" s="1" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="27" spans="23:33">
-      <c r="W27" s="19" t="s">
+    <row r="27" spans="23:33" x14ac:dyDescent="0.25">
+      <c r="W27" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="X27" s="19"/>
-      <c r="Y27" s="19"/>
-      <c r="Z27" s="19"/>
-      <c r="AA27" s="19"/>
-      <c r="AB27" s="19"/>
-      <c r="AC27" s="19"/>
-      <c r="AD27" s="19"/>
-      <c r="AE27" s="19"/>
-      <c r="AF27" s="19"/>
-      <c r="AG27" s="19"/>
-    </row>
-    <row r="28" spans="23:33">
-      <c r="W28" s="19"/>
-      <c r="X28" s="19"/>
-      <c r="Y28" s="19"/>
-      <c r="Z28" s="19"/>
-      <c r="AA28" s="19"/>
-      <c r="AB28" s="19"/>
-      <c r="AC28" s="19"/>
-      <c r="AD28" s="19"/>
-      <c r="AE28" s="19"/>
-      <c r="AF28" s="19"/>
-      <c r="AG28" s="19"/>
-    </row>
-    <row r="29" spans="23:33" ht="108" customHeight="1">
-      <c r="W29" s="19"/>
-      <c r="X29" s="19"/>
-      <c r="Y29" s="19"/>
-      <c r="Z29" s="19"/>
-      <c r="AA29" s="19"/>
-      <c r="AB29" s="19"/>
-      <c r="AC29" s="19"/>
-      <c r="AD29" s="19"/>
-      <c r="AE29" s="19"/>
-      <c r="AF29" s="19"/>
-      <c r="AG29" s="19"/>
-    </row>
-    <row r="30" spans="23:33">
-      <c r="W30" s="19"/>
-      <c r="X30" s="19"/>
-      <c r="Y30" s="19"/>
-      <c r="Z30" s="19"/>
-      <c r="AA30" s="19"/>
-      <c r="AB30" s="19"/>
-      <c r="AC30" s="19"/>
-      <c r="AD30" s="19"/>
-      <c r="AE30" s="19"/>
-      <c r="AF30" s="19"/>
-      <c r="AG30" s="19"/>
-    </row>
-    <row r="32" spans="23:33" ht="14.25" customHeight="1"/>
-    <row r="33" spans="23:42" ht="77.25" customHeight="1">
-      <c r="W33" s="19" t="s">
+      <c r="X27" s="8"/>
+      <c r="Y27" s="8"/>
+      <c r="Z27" s="8"/>
+      <c r="AA27" s="8"/>
+      <c r="AB27" s="8"/>
+      <c r="AC27" s="8"/>
+      <c r="AD27" s="8"/>
+      <c r="AE27" s="8"/>
+      <c r="AF27" s="8"/>
+      <c r="AG27" s="8"/>
+    </row>
+    <row r="28" spans="23:33" x14ac:dyDescent="0.25">
+      <c r="W28" s="8"/>
+      <c r="X28" s="8"/>
+      <c r="Y28" s="8"/>
+      <c r="Z28" s="8"/>
+      <c r="AA28" s="8"/>
+      <c r="AB28" s="8"/>
+      <c r="AC28" s="8"/>
+      <c r="AD28" s="8"/>
+      <c r="AE28" s="8"/>
+      <c r="AF28" s="8"/>
+      <c r="AG28" s="8"/>
+    </row>
+    <row r="29" spans="23:33" ht="108" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W29" s="8"/>
+      <c r="X29" s="8"/>
+      <c r="Y29" s="8"/>
+      <c r="Z29" s="8"/>
+      <c r="AA29" s="8"/>
+      <c r="AB29" s="8"/>
+      <c r="AC29" s="8"/>
+      <c r="AD29" s="8"/>
+      <c r="AE29" s="8"/>
+      <c r="AF29" s="8"/>
+      <c r="AG29" s="8"/>
+    </row>
+    <row r="30" spans="23:33" x14ac:dyDescent="0.25">
+      <c r="W30" s="8"/>
+      <c r="X30" s="8"/>
+      <c r="Y30" s="8"/>
+      <c r="Z30" s="8"/>
+      <c r="AA30" s="8"/>
+      <c r="AB30" s="8"/>
+      <c r="AC30" s="8"/>
+      <c r="AD30" s="8"/>
+      <c r="AE30" s="8"/>
+      <c r="AF30" s="8"/>
+      <c r="AG30" s="8"/>
+    </row>
+    <row r="32" spans="23:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="23:42" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W33" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="X33" s="19"/>
-      <c r="Y33" s="19"/>
-      <c r="Z33" s="19"/>
-      <c r="AA33" s="19"/>
-      <c r="AB33" s="19"/>
-      <c r="AC33" s="19"/>
-      <c r="AD33" s="19"/>
-      <c r="AE33" s="19"/>
-      <c r="AF33" s="19"/>
-      <c r="AG33" s="19"/>
-    </row>
-    <row r="35" spans="23:42">
-      <c r="W35" s="19" t="s">
+      <c r="X33" s="8"/>
+      <c r="Y33" s="8"/>
+      <c r="Z33" s="8"/>
+      <c r="AA33" s="8"/>
+      <c r="AB33" s="8"/>
+      <c r="AC33" s="8"/>
+      <c r="AD33" s="8"/>
+      <c r="AE33" s="8"/>
+      <c r="AF33" s="8"/>
+      <c r="AG33" s="8"/>
+    </row>
+    <row r="35" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W35" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="X35" s="20"/>
-      <c r="Y35" s="20"/>
-      <c r="Z35" s="20"/>
-      <c r="AA35" s="20"/>
-      <c r="AB35" s="20"/>
-      <c r="AC35" s="20"/>
-      <c r="AD35" s="20"/>
-      <c r="AE35" s="20"/>
-      <c r="AF35" s="20"/>
-      <c r="AG35" s="20"/>
-      <c r="AI35" s="23" t="s">
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
+      <c r="AC35" s="9"/>
+      <c r="AD35" s="9"/>
+      <c r="AE35" s="9"/>
+      <c r="AF35" s="9"/>
+      <c r="AG35" s="9"/>
+      <c r="AI35" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="AJ35" s="21"/>
-      <c r="AK35" s="21"/>
-      <c r="AL35" s="21"/>
-      <c r="AM35" s="21"/>
-      <c r="AN35" s="21"/>
-      <c r="AO35" s="21"/>
-      <c r="AP35" s="21"/>
-    </row>
-    <row r="36" spans="23:42">
-      <c r="W36" s="20"/>
-      <c r="X36" s="20"/>
-      <c r="Y36" s="20"/>
-      <c r="Z36" s="20"/>
-      <c r="AA36" s="20"/>
-      <c r="AB36" s="20"/>
-      <c r="AC36" s="20"/>
-      <c r="AD36" s="20"/>
-      <c r="AE36" s="20"/>
-      <c r="AF36" s="20"/>
-      <c r="AG36" s="20"/>
-      <c r="AI36" s="21"/>
-      <c r="AJ36" s="21"/>
-      <c r="AK36" s="21"/>
-      <c r="AL36" s="21"/>
-      <c r="AM36" s="21"/>
-      <c r="AN36" s="21"/>
-      <c r="AO36" s="21"/>
-      <c r="AP36" s="21"/>
-    </row>
-    <row r="37" spans="23:42">
-      <c r="W37" s="20"/>
-      <c r="X37" s="20"/>
-      <c r="Y37" s="20"/>
-      <c r="Z37" s="20"/>
-      <c r="AA37" s="20"/>
-      <c r="AB37" s="20"/>
-      <c r="AC37" s="20"/>
-      <c r="AD37" s="20"/>
-      <c r="AE37" s="20"/>
-      <c r="AF37" s="20"/>
-      <c r="AG37" s="20"/>
-      <c r="AI37" s="21"/>
-      <c r="AJ37" s="21"/>
-      <c r="AK37" s="21"/>
-      <c r="AL37" s="21"/>
-      <c r="AM37" s="21"/>
-      <c r="AN37" s="21"/>
-      <c r="AO37" s="21"/>
-      <c r="AP37" s="21"/>
-    </row>
-    <row r="38" spans="23:42">
-      <c r="W38" s="20"/>
-      <c r="X38" s="20"/>
-      <c r="Y38" s="20"/>
-      <c r="Z38" s="20"/>
-      <c r="AA38" s="20"/>
-      <c r="AB38" s="20"/>
-      <c r="AC38" s="20"/>
-      <c r="AD38" s="20"/>
-      <c r="AE38" s="20"/>
-      <c r="AF38" s="20"/>
-      <c r="AG38" s="20"/>
-      <c r="AI38" s="21"/>
-      <c r="AJ38" s="21"/>
-      <c r="AK38" s="21"/>
-      <c r="AL38" s="21"/>
-      <c r="AM38" s="21"/>
-      <c r="AN38" s="21"/>
-      <c r="AO38" s="21"/>
-      <c r="AP38" s="21"/>
-    </row>
-    <row r="39" spans="23:42">
-      <c r="W39" s="20"/>
-      <c r="X39" s="20"/>
-      <c r="Y39" s="20"/>
-      <c r="Z39" s="20"/>
-      <c r="AA39" s="20"/>
-      <c r="AB39" s="20"/>
-      <c r="AC39" s="20"/>
-      <c r="AD39" s="20"/>
-      <c r="AE39" s="20"/>
-      <c r="AF39" s="20"/>
-      <c r="AG39" s="20"/>
-      <c r="AI39" s="21"/>
-      <c r="AJ39" s="21"/>
-      <c r="AK39" s="21"/>
-      <c r="AL39" s="21"/>
-      <c r="AM39" s="21"/>
-      <c r="AN39" s="21"/>
-      <c r="AO39" s="21"/>
-      <c r="AP39" s="21"/>
-    </row>
-    <row r="40" spans="23:42">
-      <c r="W40" s="20"/>
-      <c r="X40" s="20"/>
-      <c r="Y40" s="20"/>
-      <c r="Z40" s="20"/>
-      <c r="AA40" s="20"/>
-      <c r="AB40" s="20"/>
-      <c r="AC40" s="20"/>
-      <c r="AD40" s="20"/>
-      <c r="AE40" s="20"/>
-      <c r="AF40" s="20"/>
-      <c r="AG40" s="20"/>
-      <c r="AI40" s="21"/>
-      <c r="AJ40" s="21"/>
-      <c r="AK40" s="21"/>
-      <c r="AL40" s="21"/>
-      <c r="AM40" s="21"/>
-      <c r="AN40" s="21"/>
-      <c r="AO40" s="21"/>
-      <c r="AP40" s="21"/>
-    </row>
-    <row r="41" spans="23:42">
-      <c r="W41" s="20"/>
-      <c r="X41" s="20"/>
-      <c r="Y41" s="20"/>
-      <c r="Z41" s="20"/>
-      <c r="AA41" s="20"/>
-      <c r="AB41" s="20"/>
-      <c r="AC41" s="20"/>
-      <c r="AD41" s="20"/>
-      <c r="AE41" s="20"/>
-      <c r="AF41" s="20"/>
-      <c r="AG41" s="20"/>
-      <c r="AI41" s="21"/>
-      <c r="AJ41" s="21"/>
-      <c r="AK41" s="21"/>
-      <c r="AL41" s="21"/>
-      <c r="AM41" s="21"/>
-      <c r="AN41" s="21"/>
-      <c r="AO41" s="21"/>
-      <c r="AP41" s="21"/>
-    </row>
-    <row r="42" spans="23:42" ht="78" customHeight="1">
-      <c r="W42" s="20"/>
-      <c r="X42" s="20"/>
-      <c r="Y42" s="20"/>
-      <c r="Z42" s="20"/>
-      <c r="AA42" s="20"/>
-      <c r="AB42" s="20"/>
-      <c r="AC42" s="20"/>
-      <c r="AD42" s="20"/>
-      <c r="AE42" s="20"/>
-      <c r="AF42" s="20"/>
-      <c r="AG42" s="20"/>
-      <c r="AI42" s="21"/>
-      <c r="AJ42" s="21"/>
-      <c r="AK42" s="21"/>
-      <c r="AL42" s="21"/>
-      <c r="AM42" s="21"/>
-      <c r="AN42" s="21"/>
-      <c r="AO42" s="21"/>
-      <c r="AP42" s="21"/>
-    </row>
-    <row r="48" spans="23:42" ht="136.5" customHeight="1"/>
+      <c r="AJ35" s="11"/>
+      <c r="AK35" s="11"/>
+      <c r="AL35" s="11"/>
+      <c r="AM35" s="11"/>
+      <c r="AN35" s="11"/>
+      <c r="AO35" s="11"/>
+      <c r="AP35" s="11"/>
+    </row>
+    <row r="36" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="9"/>
+      <c r="AB36" s="9"/>
+      <c r="AC36" s="9"/>
+      <c r="AD36" s="9"/>
+      <c r="AE36" s="9"/>
+      <c r="AF36" s="9"/>
+      <c r="AG36" s="9"/>
+      <c r="AI36" s="11"/>
+      <c r="AJ36" s="11"/>
+      <c r="AK36" s="11"/>
+      <c r="AL36" s="11"/>
+      <c r="AM36" s="11"/>
+      <c r="AN36" s="11"/>
+      <c r="AO36" s="11"/>
+      <c r="AP36" s="11"/>
+    </row>
+    <row r="37" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W37" s="9"/>
+      <c r="X37" s="9"/>
+      <c r="Y37" s="9"/>
+      <c r="Z37" s="9"/>
+      <c r="AA37" s="9"/>
+      <c r="AB37" s="9"/>
+      <c r="AC37" s="9"/>
+      <c r="AD37" s="9"/>
+      <c r="AE37" s="9"/>
+      <c r="AF37" s="9"/>
+      <c r="AG37" s="9"/>
+      <c r="AI37" s="11"/>
+      <c r="AJ37" s="11"/>
+      <c r="AK37" s="11"/>
+      <c r="AL37" s="11"/>
+      <c r="AM37" s="11"/>
+      <c r="AN37" s="11"/>
+      <c r="AO37" s="11"/>
+      <c r="AP37" s="11"/>
+    </row>
+    <row r="38" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W38" s="9"/>
+      <c r="X38" s="9"/>
+      <c r="Y38" s="9"/>
+      <c r="Z38" s="9"/>
+      <c r="AA38" s="9"/>
+      <c r="AB38" s="9"/>
+      <c r="AC38" s="9"/>
+      <c r="AD38" s="9"/>
+      <c r="AE38" s="9"/>
+      <c r="AF38" s="9"/>
+      <c r="AG38" s="9"/>
+      <c r="AI38" s="11"/>
+      <c r="AJ38" s="11"/>
+      <c r="AK38" s="11"/>
+      <c r="AL38" s="11"/>
+      <c r="AM38" s="11"/>
+      <c r="AN38" s="11"/>
+      <c r="AO38" s="11"/>
+      <c r="AP38" s="11"/>
+    </row>
+    <row r="39" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W39" s="9"/>
+      <c r="X39" s="9"/>
+      <c r="Y39" s="9"/>
+      <c r="Z39" s="9"/>
+      <c r="AA39" s="9"/>
+      <c r="AB39" s="9"/>
+      <c r="AC39" s="9"/>
+      <c r="AD39" s="9"/>
+      <c r="AE39" s="9"/>
+      <c r="AF39" s="9"/>
+      <c r="AG39" s="9"/>
+      <c r="AI39" s="11"/>
+      <c r="AJ39" s="11"/>
+      <c r="AK39" s="11"/>
+      <c r="AL39" s="11"/>
+      <c r="AM39" s="11"/>
+      <c r="AN39" s="11"/>
+      <c r="AO39" s="11"/>
+      <c r="AP39" s="11"/>
+    </row>
+    <row r="40" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W40" s="9"/>
+      <c r="X40" s="9"/>
+      <c r="Y40" s="9"/>
+      <c r="Z40" s="9"/>
+      <c r="AA40" s="9"/>
+      <c r="AB40" s="9"/>
+      <c r="AC40" s="9"/>
+      <c r="AD40" s="9"/>
+      <c r="AE40" s="9"/>
+      <c r="AF40" s="9"/>
+      <c r="AG40" s="9"/>
+      <c r="AI40" s="11"/>
+      <c r="AJ40" s="11"/>
+      <c r="AK40" s="11"/>
+      <c r="AL40" s="11"/>
+      <c r="AM40" s="11"/>
+      <c r="AN40" s="11"/>
+      <c r="AO40" s="11"/>
+      <c r="AP40" s="11"/>
+    </row>
+    <row r="41" spans="23:42" x14ac:dyDescent="0.25">
+      <c r="W41" s="9"/>
+      <c r="X41" s="9"/>
+      <c r="Y41" s="9"/>
+      <c r="Z41" s="9"/>
+      <c r="AA41" s="9"/>
+      <c r="AB41" s="9"/>
+      <c r="AC41" s="9"/>
+      <c r="AD41" s="9"/>
+      <c r="AE41" s="9"/>
+      <c r="AF41" s="9"/>
+      <c r="AG41" s="9"/>
+      <c r="AI41" s="11"/>
+      <c r="AJ41" s="11"/>
+      <c r="AK41" s="11"/>
+      <c r="AL41" s="11"/>
+      <c r="AM41" s="11"/>
+      <c r="AN41" s="11"/>
+      <c r="AO41" s="11"/>
+      <c r="AP41" s="11"/>
+    </row>
+    <row r="42" spans="23:42" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="W42" s="9"/>
+      <c r="X42" s="9"/>
+      <c r="Y42" s="9"/>
+      <c r="Z42" s="9"/>
+      <c r="AA42" s="9"/>
+      <c r="AB42" s="9"/>
+      <c r="AC42" s="9"/>
+      <c r="AD42" s="9"/>
+      <c r="AE42" s="9"/>
+      <c r="AF42" s="9"/>
+      <c r="AG42" s="9"/>
+      <c r="AI42" s="11"/>
+      <c r="AJ42" s="11"/>
+      <c r="AK42" s="11"/>
+      <c r="AL42" s="11"/>
+      <c r="AM42" s="11"/>
+      <c r="AN42" s="11"/>
+      <c r="AO42" s="11"/>
+      <c r="AP42" s="11"/>
+    </row>
+    <row r="48" spans="23:42" ht="136.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="W27:AG30"/>

</xml_diff>